<commit_message>
Added support for all relevant fields, added testing, added detailed validation logic
</commit_message>
<xml_diff>
--- a/TCG Blank Model Template 2026-04-26.xlsx
+++ b/TCG Blank Model Template 2026-04-26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2434ef0feffdd206/Documents/Tryon Capital Group/Origination ^0 Due Diligence/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="735" documentId="13_ncr:1_{AF47EFD1-DEF7-4D96-959F-C8937757AD83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F298FF68-9E71-4883-BC70-24D4BF22FA5D}"/>
+  <xr:revisionPtr revIDLastSave="739" documentId="13_ncr:1_{AF47EFD1-DEF7-4D96-959F-C8937757AD83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C50B14D-466A-42FD-9D20-0A8DA9F9853B}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Deal Sheet" sheetId="15" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <definedName name="Am_Sched_Mnthly">'Amortization Schedule - Monthly'!$B$3:$F$362</definedName>
     <definedName name="Am_Sched_Mnthly_Mnths">'Amortization Schedule - Monthly'!$B$3:$B$362</definedName>
     <definedName name="AskingPrice">'Inputs &amp; Summary'!$D$7</definedName>
+    <definedName name="AssessedValue">'Inputs &amp; Summary'!$D$70</definedName>
     <definedName name="Bathrooms">'Inputs &amp; Summary'!$D$9</definedName>
     <definedName name="Bedrooms">'Inputs &amp; Summary'!$D$8</definedName>
     <definedName name="ExpenseGrowth">'Inputs &amp; Summary'!$D$96</definedName>
@@ -1759,9 +1760,6 @@
     <t>Stabalization Month</t>
   </si>
   <si>
-    <t>Rehab &amp; Contingency</t>
-  </si>
-  <si>
     <t>Price/SF</t>
   </si>
   <si>
@@ -1973,6 +1971,9 @@
   </si>
   <si>
     <t>All-In Transaction Size</t>
+  </si>
+  <si>
+    <t>Initial Rehab &amp; Contingency</t>
   </si>
 </sst>
 </file>
@@ -3231,7 +3232,7 @@
         <v>88</v>
       </c>
       <c r="E4" s="79" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G4" s="78" t="s">
         <v>37</v>
@@ -3906,7 +3907,7 @@
       <c r="O2" s="157"/>
       <c r="P2" s="158"/>
       <c r="R2" s="160" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="S2" s="161"/>
       <c r="T2" s="161"/>
@@ -3945,13 +3946,13 @@
         <v>74</v>
       </c>
       <c r="R3" s="134" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="U3" s="134" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="V3" s="134" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
@@ -3990,19 +3991,19 @@
       </c>
       <c r="P4" s="197"/>
       <c r="R4" s="134" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="S4" s="134" t="s">
+        <v>201</v>
+      </c>
+      <c r="T4" s="134" t="s">
         <v>202</v>
       </c>
-      <c r="T4" s="134" t="s">
-        <v>203</v>
-      </c>
       <c r="U4" s="134" t="s">
+        <v>222</v>
+      </c>
+      <c r="V4" s="134" t="s">
         <v>223</v>
-      </c>
-      <c r="V4" s="134" t="s">
-        <v>224</v>
       </c>
       <c r="W4" s="134" t="s">
         <v>81</v>
@@ -4016,7 +4017,7 @@
         <v>120</v>
       </c>
       <c r="D5" s="125" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F5" s="14" t="s">
         <v>3</v>
@@ -4055,13 +4056,13 @@
         <v>0</v>
       </c>
       <c r="U5" s="172" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V5" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W5" s="149" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
@@ -4096,13 +4097,13 @@
         <v>1230</v>
       </c>
       <c r="U6" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V6" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W6" s="149" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
@@ -4155,13 +4156,13 @@
         <v>3128</v>
       </c>
       <c r="U7" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V7" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W7" s="149" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
@@ -4212,13 +4213,13 @@
         <v>5027</v>
       </c>
       <c r="U8" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V8" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W8" s="149" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4272,13 +4273,13 @@
         <v>6925</v>
       </c>
       <c r="U9" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V9" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W9" s="149" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
@@ -4314,13 +4315,13 @@
         <v>8824</v>
       </c>
       <c r="U10" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V10" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W10" s="149" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4369,13 +4370,13 @@
         <v>10798</v>
       </c>
       <c r="U11" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V11" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W11" s="149" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
@@ -4427,13 +4428,13 @@
         <v>13051</v>
       </c>
       <c r="U12" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V12" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W12" s="149" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
@@ -4477,13 +4478,13 @@
         <v>15536</v>
       </c>
       <c r="U13" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V13" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W13" s="149" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
@@ -4516,7 +4517,7 @@
         <v>n/a</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="P14" s="47" t="str">
         <f>IFERROR(D17-P12, "n/a")</f>
@@ -4532,13 +4533,13 @@
         <v>18463</v>
       </c>
       <c r="U14" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V14" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W14" s="149" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
@@ -4566,7 +4567,7 @@
         <v>-0.08</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="P15" s="47" t="str">
         <f>IFERROR(D47+D40+D49, "n/a")</f>
@@ -4583,13 +4584,13 @@
         <v>21627</v>
       </c>
       <c r="U15" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="V15" s="136" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W15" s="149" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="16" spans="1:25" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4628,12 +4629,12 @@
         <v>n/a</v>
       </c>
       <c r="R16" s="194" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="S16" s="194"/>
       <c r="T16" s="194"/>
       <c r="W16" s="194" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="X16" s="194"/>
       <c r="Y16" s="194"/>
@@ -4671,7 +4672,7 @@
         <v>n/a</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="P17" s="47" t="str">
         <f>IFERROR((D21-D27)*D17, "n/a")</f>
@@ -4693,7 +4694,7 @@
         <v>n/a</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G18" s="13">
         <f>-D92</f>
@@ -4704,7 +4705,7 @@
         <v>n/a</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K18" s="181">
         <f ca="1">IFERROR(INDEX('Monthly Proforma'!E21:DT21, MATCH($K$2, 'Monthly Proforma'!E$8:DT$8, 0)), "n/a")</f>
@@ -4715,7 +4716,7 @@
         <v>n/a</v>
       </c>
       <c r="N18" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="O18" s="8"/>
       <c r="P18" s="190">
@@ -4731,7 +4732,7 @@
     </row>
     <row r="19" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D19" s="133" t="str">
         <f>IFERROR(D17/D10, "n/a")</f>
@@ -4760,7 +4761,7 @@
         <v>n/a</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="P19" s="191">
         <f>IFERROR(SUM(P14:P18), "n/a")</f>
@@ -4782,7 +4783,7 @@
       </c>
       <c r="D20" s="125">
         <f ca="1">TODAY()+30</f>
-        <v>46170</v>
+        <v>46174</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>19</v>
@@ -4806,13 +4807,13 @@
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D21" s="21">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G21" s="177" t="str">
         <f ca="1">IFERROR(G19+G20, "n/a")</f>
@@ -4820,7 +4821,7 @@
       </c>
       <c r="H21" s="119"/>
       <c r="J21" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K21" s="177" t="str">
         <f ca="1">IFERROR(K19+K20, "n/a")</f>
@@ -4828,7 +4829,7 @@
       </c>
       <c r="L21" s="119"/>
       <c r="N21" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="O21" s="8"/>
       <c r="P21" s="162">
@@ -4839,27 +4840,27 @@
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D22" s="46" t="s">
         <v>43</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="G22" s="150" t="str">
         <f ca="1">IFERROR((G8+G13+G14+G15+G16+G18)+G20, "n/a")</f>
         <v>n/a</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="K22" s="150" t="str">
         <f ca="1">IFERROR((K8+K13+K14+K15+K16+K18)+K20, "n/a")</f>
         <v>n/a</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="P22" s="191">
         <f>IFERROR(SUM(P14:P18)+P21, "n/a")</f>
@@ -4875,7 +4876,7 @@
         <v>n/a</v>
       </c>
       <c r="N23" s="6" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="P23" s="133" t="str">
         <f>IFERROR(LoanAmount+P22, "n/a")</f>
@@ -4884,7 +4885,7 @@
     </row>
     <row r="24" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F24" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G24" s="173" t="str">
         <f ca="1">IFERROR(G19/-G20, "n/a")</f>
@@ -4892,7 +4893,7 @@
       </c>
       <c r="H24" s="22"/>
       <c r="J24" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K24" s="173" t="str">
         <f ca="1">IFERROR(K19/-K20, "n/a")</f>
@@ -4907,7 +4908,7 @@
       <c r="C25" s="193"/>
       <c r="D25" s="193"/>
       <c r="F25" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G25" s="173" t="str">
         <f ca="1">IFERROR((G8+G13+G14)/-G20, "n/a")</f>
@@ -4915,7 +4916,7 @@
       </c>
       <c r="H25" s="22"/>
       <c r="J25" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K25" s="173" t="str">
         <f ca="1">IFERROR((K8+K13+K14)/-K20, "n/a")</f>
@@ -4940,21 +4941,21 @@
         <v>0</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G26" s="137" t="str">
         <f ca="1">IFERROR((G21*12)/$P$22, "n/a")</f>
         <v>n/a</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="K26" s="137" t="str">
         <f ca="1">IFERROR((K21*12)/$P$22, "n/a")</f>
         <v>n/a</v>
       </c>
       <c r="N26" s="195" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="O26" s="195"/>
       <c r="P26" s="195"/>
@@ -4964,20 +4965,20 @@
         <v>133</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D27" s="21">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G27" s="137" t="str">
         <f ca="1">IFERROR((G22*12)/$P$22, "n/a")</f>
         <v>n/a</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="K27" s="137" t="str">
         <f ca="1">IFERROR((K22*12)/$P$22, "n/a")</f>
@@ -4992,7 +4993,7 @@
         <v>133</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D28" s="126">
         <v>0</v>
@@ -5014,7 +5015,7 @@
         <v>n/a</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G29" s="137" t="str">
         <f ca="1">IFERROR((G19*12)/$D$17, "n/a")</f>
@@ -5025,7 +5026,7 @@
         <v>n/a</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="K29" s="137" t="str">
         <f ca="1">IFERROR((K19*12)/$D$17, "n/a")</f>
@@ -5114,7 +5115,7 @@
         <v>46</v>
       </c>
       <c r="D34" s="20">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="N34" s="195"/>
       <c r="O34" s="195"/>
@@ -5153,9 +5154,9 @@
         <v>133</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="D37" s="46" t="str">
+        <v>200</v>
+      </c>
+      <c r="D37" s="176" t="str">
         <f>IFERROR((T13/R13)/LoanAmount, "n/a")</f>
         <v>n/a</v>
       </c>
@@ -5257,7 +5258,7 @@
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B46" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D46" s="21">
         <f>8535/506250</f>
@@ -5269,7 +5270,7 @@
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B47" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D47" s="133" t="str">
         <f>IFERROR(P12*D46, "n/a")</f>
@@ -5284,7 +5285,7 @@
         <v>133</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D48" s="4">
         <v>5</v>
@@ -5295,7 +5296,7 @@
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B49" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D49" s="133">
         <f>1495+695+1000+300+(D48*350)</f>
@@ -5326,7 +5327,7 @@
         <v>133</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>174</v>
+        <v>245</v>
       </c>
       <c r="D52" s="3">
         <v>250</v>
@@ -5395,7 +5396,7 @@
         <v>133</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D58" s="126" t="s">
         <v>135</v>
@@ -5409,7 +5410,7 @@
         <v>133</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D59" s="126" t="s">
         <v>135</v>
@@ -5423,7 +5424,7 @@
         <v>133</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D60" s="126" t="s">
         <v>135</v>
@@ -5437,7 +5438,7 @@
         <v>133</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D61" s="126" t="s">
         <v>135</v>
@@ -5451,7 +5452,7 @@
         <v>133</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D62" s="126" t="s">
         <v>135</v>
@@ -5476,7 +5477,7 @@
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A64" s="1"/>
       <c r="B64" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D64" s="138" t="str">
         <f>IFERROR(D63/D10,"n/a")</f>
@@ -5489,7 +5490,7 @@
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A65" s="1"/>
       <c r="B65" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D65" s="137" t="str">
         <f>IFERROR(D63/P23, "n/a")</f>
@@ -5547,7 +5548,7 @@
         <v>133</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D70" s="126" t="s">
         <v>135</v>
@@ -5561,7 +5562,7 @@
         <v>133</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D71" s="4">
         <v>2027</v>
@@ -5575,7 +5576,7 @@
         <v>133</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D72" s="122">
         <v>4</v>
@@ -5624,7 +5625,7 @@
     </row>
     <row r="77" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B77" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D77" s="132">
         <v>0.65</v>
@@ -5635,7 +5636,7 @@
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B78" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D78" s="174" t="str">
         <f>IFERROR(MIN(0.3, (0.1*LN($D$11))), "n/a")</f>
@@ -5647,7 +5648,7 @@
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B79" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D79" s="174" t="str">
         <f ca="1">IFERROR(MIN(0.3, (0.15*((YEAR(TODAY())-$D$6)/40))), "n/a")</f>
@@ -5662,7 +5663,7 @@
         <v>133</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D80" s="144">
         <v>0</v>
@@ -5678,7 +5679,7 @@
     </row>
     <row r="82" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B82" s="193" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C82" s="193"/>
       <c r="D82" s="193"/>
@@ -5691,7 +5692,7 @@
         <v>133</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D83" s="132">
         <v>0.8</v>
@@ -5705,7 +5706,7 @@
         <v>133</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D84" s="126">
         <v>250</v>
@@ -5716,7 +5717,7 @@
     </row>
     <row r="85" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B85" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D85" s="138" t="str">
         <f>IFERROR(-(G17*12)/D10, "n/a")</f>
@@ -5760,7 +5761,7 @@
         <v>133</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D89" s="16">
         <v>0.08</v>
@@ -5797,7 +5798,7 @@
     </row>
     <row r="92" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B92" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D92" s="126">
         <v>0</v>
@@ -5814,7 +5815,7 @@
     </row>
     <row r="94" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B94" s="193" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C94" s="193"/>
       <c r="D94" s="193"/>
@@ -5827,7 +5828,7 @@
         <v>133</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D95" s="21">
         <v>2.5000000000000001E-2</v>
@@ -5869,7 +5870,7 @@
         <v>133</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D98" s="21">
         <v>0.04</v>
@@ -5883,7 +5884,7 @@
         <v>133</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D99" s="21">
         <v>7.4999999999999997E-3</v>
@@ -5951,7 +5952,7 @@
         <v>133</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D105" s="21">
         <f>0.05 + 0.015 + 0 + 0.005</f>
@@ -5980,7 +5981,7 @@
     </row>
     <row r="108" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B108" s="151" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="N108" s="195"/>
       <c r="O108" s="195"/>
@@ -6009,7 +6010,7 @@
     </row>
     <row r="111" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B111" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D111" s="117">
         <f>D110/12</f>
@@ -6106,7 +6107,7 @@
     </row>
     <row r="121" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B121" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D121" s="133" t="str">
         <f>IFERROR(PMT(D119/12,D120*12,-D116), "n/a")</f>
@@ -6253,11 +6254,11 @@
   <sheetData>
     <row r="1" spans="2:124" x14ac:dyDescent="0.25">
       <c r="C1" s="153" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D1" s="155" cm="1">
         <f t="array" aca="1" ref="D1" ca="1">INDEX(E8:DT8, MATCH(1, ('Inputs &amp; Summary'!D71=YEAR(E6:DT6))*(1=MONTH(E6:DT6)), 0))</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E1" s="171" t="str">
         <f t="shared" ref="E1:AJ1" ca="1" si="0">IF(MOD(E$8-$D$1, (ReassessmentFreq*12))=0, "x", "")</f>
@@ -6285,11 +6286,11 @@
       </c>
       <c r="K1" s="171" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="L1" s="171" t="str">
         <f t="shared" ca="1" si="0"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="M1" s="171" t="str">
         <f t="shared" ca="1" si="0"/>
@@ -6477,11 +6478,11 @@
       </c>
       <c r="BG1" s="171" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="BH1" s="171" t="str">
         <f t="shared" ca="1" si="1"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="BI1" s="171" t="str">
         <f t="shared" ca="1" si="1"/>
@@ -6669,11 +6670,11 @@
       </c>
       <c r="DC1" s="171" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v/>
+        <v>x</v>
       </c>
       <c r="DD1" s="171" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>x</v>
+        <v/>
       </c>
       <c r="DE1" s="171" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -6742,7 +6743,7 @@
     </row>
     <row r="2" spans="2:124" x14ac:dyDescent="0.25">
       <c r="C2" s="153" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D2" s="154" t="str">
         <f>'Inputs &amp; Summary'!D70</f>
@@ -6772,9 +6773,9 @@
         <f t="shared" ca="1" si="4"/>
         <v>$x</v>
       </c>
-      <c r="K2" s="154" t="str">
+      <c r="K2" s="154">
         <f t="shared" ca="1" si="4"/>
-        <v>$x</v>
+        <v>0</v>
       </c>
       <c r="L2" s="154">
         <f t="shared" ca="1" si="4"/>
@@ -7263,7 +7264,7 @@
       </c>
       <c r="K3" s="156">
         <f t="shared" ca="1" si="8"/>
-        <v>7.7</v>
+        <v>7.9336117681132841</v>
       </c>
       <c r="L3" s="156">
         <f t="shared" ca="1" si="8"/>
@@ -7455,7 +7456,7 @@
       </c>
       <c r="BG3" s="156">
         <f t="shared" ca="1" si="9"/>
-        <v>7.9336117681132841</v>
+        <v>8.1743111282007259</v>
       </c>
       <c r="BH3" s="156">
         <f t="shared" ca="1" si="9"/>
@@ -7647,7 +7648,7 @@
       </c>
       <c r="DC3" s="156">
         <f t="shared" ca="1" si="11"/>
-        <v>8.1743111282007259</v>
+        <v>8.4223131120665791</v>
       </c>
       <c r="DD3" s="156">
         <f t="shared" ca="1" si="11"/>
@@ -7720,7 +7721,7 @@
     </row>
     <row r="4" spans="2:124" x14ac:dyDescent="0.25">
       <c r="C4" s="153" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E4" s="171" t="str">
         <f>IF(AND(MOD(E$8-13, 12)=0, E$8&gt;=13), "x", "")</f>
@@ -8205,7 +8206,7 @@
     </row>
     <row r="5" spans="2:124" x14ac:dyDescent="0.25">
       <c r="C5" s="153" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D5" s="155">
         <f>'Inputs &amp; Summary'!D57</f>
@@ -8698,487 +8699,487 @@
       </c>
       <c r="D6" s="24">
         <f ca="1">'Inputs &amp; Summary'!$D$20</f>
-        <v>46170</v>
+        <v>46174</v>
       </c>
       <c r="E6" s="24">
         <f ca="1">EOMONTH(D6,1)</f>
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="F6" s="24">
         <f t="shared" ref="F6:BQ6" ca="1" si="16">EOMONTH(E6,1)</f>
-        <v>46234</v>
+        <v>46265</v>
       </c>
       <c r="G6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46265</v>
+        <v>46295</v>
       </c>
       <c r="H6" s="24">
         <f ca="1">EOMONTH(G6,1)</f>
-        <v>46295</v>
+        <v>46326</v>
       </c>
       <c r="I6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46326</v>
+        <v>46356</v>
       </c>
       <c r="J6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46356</v>
+        <v>46387</v>
       </c>
       <c r="K6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46387</v>
+        <v>46418</v>
       </c>
       <c r="L6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46418</v>
+        <v>46446</v>
       </c>
       <c r="M6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46446</v>
+        <v>46477</v>
       </c>
       <c r="N6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46477</v>
+        <v>46507</v>
       </c>
       <c r="O6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46507</v>
+        <v>46538</v>
       </c>
       <c r="P6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46538</v>
+        <v>46568</v>
       </c>
       <c r="Q6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46568</v>
+        <v>46599</v>
       </c>
       <c r="R6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46599</v>
+        <v>46630</v>
       </c>
       <c r="S6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46630</v>
+        <v>46660</v>
       </c>
       <c r="T6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46660</v>
+        <v>46691</v>
       </c>
       <c r="U6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46691</v>
+        <v>46721</v>
       </c>
       <c r="V6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46721</v>
+        <v>46752</v>
       </c>
       <c r="W6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46752</v>
+        <v>46783</v>
       </c>
       <c r="X6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46783</v>
+        <v>46812</v>
       </c>
       <c r="Y6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46812</v>
+        <v>46843</v>
       </c>
       <c r="Z6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46843</v>
+        <v>46873</v>
       </c>
       <c r="AA6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46873</v>
+        <v>46904</v>
       </c>
       <c r="AB6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46904</v>
+        <v>46934</v>
       </c>
       <c r="AC6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46934</v>
+        <v>46965</v>
       </c>
       <c r="AD6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46965</v>
+        <v>46996</v>
       </c>
       <c r="AE6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>46996</v>
+        <v>47026</v>
       </c>
       <c r="AF6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47026</v>
+        <v>47057</v>
       </c>
       <c r="AG6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47057</v>
+        <v>47087</v>
       </c>
       <c r="AH6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47087</v>
+        <v>47118</v>
       </c>
       <c r="AI6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47118</v>
+        <v>47149</v>
       </c>
       <c r="AJ6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47149</v>
+        <v>47177</v>
       </c>
       <c r="AK6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47177</v>
+        <v>47208</v>
       </c>
       <c r="AL6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47208</v>
+        <v>47238</v>
       </c>
       <c r="AM6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47238</v>
+        <v>47269</v>
       </c>
       <c r="AN6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47269</v>
+        <v>47299</v>
       </c>
       <c r="AO6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47299</v>
+        <v>47330</v>
       </c>
       <c r="AP6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47330</v>
+        <v>47361</v>
       </c>
       <c r="AQ6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47361</v>
+        <v>47391</v>
       </c>
       <c r="AR6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47391</v>
+        <v>47422</v>
       </c>
       <c r="AS6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47422</v>
+        <v>47452</v>
       </c>
       <c r="AT6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47452</v>
+        <v>47483</v>
       </c>
       <c r="AU6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47483</v>
+        <v>47514</v>
       </c>
       <c r="AV6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47514</v>
+        <v>47542</v>
       </c>
       <c r="AW6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47542</v>
+        <v>47573</v>
       </c>
       <c r="AX6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47573</v>
+        <v>47603</v>
       </c>
       <c r="AY6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47603</v>
+        <v>47634</v>
       </c>
       <c r="AZ6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47634</v>
+        <v>47664</v>
       </c>
       <c r="BA6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47664</v>
+        <v>47695</v>
       </c>
       <c r="BB6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47695</v>
+        <v>47726</v>
       </c>
       <c r="BC6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47726</v>
+        <v>47756</v>
       </c>
       <c r="BD6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47756</v>
+        <v>47787</v>
       </c>
       <c r="BE6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47787</v>
+        <v>47817</v>
       </c>
       <c r="BF6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47817</v>
+        <v>47848</v>
       </c>
       <c r="BG6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47848</v>
+        <v>47879</v>
       </c>
       <c r="BH6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47879</v>
+        <v>47907</v>
       </c>
       <c r="BI6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47907</v>
+        <v>47938</v>
       </c>
       <c r="BJ6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47938</v>
+        <v>47968</v>
       </c>
       <c r="BK6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47968</v>
+        <v>47999</v>
       </c>
       <c r="BL6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>47999</v>
+        <v>48029</v>
       </c>
       <c r="BM6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>48029</v>
+        <v>48060</v>
       </c>
       <c r="BN6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>48060</v>
+        <v>48091</v>
       </c>
       <c r="BO6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>48091</v>
+        <v>48121</v>
       </c>
       <c r="BP6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>48121</v>
+        <v>48152</v>
       </c>
       <c r="BQ6" s="24">
         <f t="shared" ca="1" si="16"/>
-        <v>48152</v>
+        <v>48182</v>
       </c>
       <c r="BR6" s="24">
         <f t="shared" ref="BR6:DT6" ca="1" si="17">EOMONTH(BQ6,1)</f>
-        <v>48182</v>
+        <v>48213</v>
       </c>
       <c r="BS6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48213</v>
+        <v>48244</v>
       </c>
       <c r="BT6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48244</v>
+        <v>48273</v>
       </c>
       <c r="BU6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48273</v>
+        <v>48304</v>
       </c>
       <c r="BV6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48304</v>
+        <v>48334</v>
       </c>
       <c r="BW6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48334</v>
+        <v>48365</v>
       </c>
       <c r="BX6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48365</v>
+        <v>48395</v>
       </c>
       <c r="BY6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48395</v>
+        <v>48426</v>
       </c>
       <c r="BZ6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48426</v>
+        <v>48457</v>
       </c>
       <c r="CA6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48457</v>
+        <v>48487</v>
       </c>
       <c r="CB6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48487</v>
+        <v>48518</v>
       </c>
       <c r="CC6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48518</v>
+        <v>48548</v>
       </c>
       <c r="CD6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48548</v>
+        <v>48579</v>
       </c>
       <c r="CE6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48579</v>
+        <v>48610</v>
       </c>
       <c r="CF6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48610</v>
+        <v>48638</v>
       </c>
       <c r="CG6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48638</v>
+        <v>48669</v>
       </c>
       <c r="CH6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48669</v>
+        <v>48699</v>
       </c>
       <c r="CI6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48699</v>
+        <v>48730</v>
       </c>
       <c r="CJ6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48730</v>
+        <v>48760</v>
       </c>
       <c r="CK6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48760</v>
+        <v>48791</v>
       </c>
       <c r="CL6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48791</v>
+        <v>48822</v>
       </c>
       <c r="CM6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48822</v>
+        <v>48852</v>
       </c>
       <c r="CN6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48852</v>
+        <v>48883</v>
       </c>
       <c r="CO6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48883</v>
+        <v>48913</v>
       </c>
       <c r="CP6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48913</v>
+        <v>48944</v>
       </c>
       <c r="CQ6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48944</v>
+        <v>48975</v>
       </c>
       <c r="CR6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>48975</v>
+        <v>49003</v>
       </c>
       <c r="CS6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49003</v>
+        <v>49034</v>
       </c>
       <c r="CT6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49034</v>
+        <v>49064</v>
       </c>
       <c r="CU6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49064</v>
+        <v>49095</v>
       </c>
       <c r="CV6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49095</v>
+        <v>49125</v>
       </c>
       <c r="CW6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49125</v>
+        <v>49156</v>
       </c>
       <c r="CX6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49156</v>
+        <v>49187</v>
       </c>
       <c r="CY6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49187</v>
+        <v>49217</v>
       </c>
       <c r="CZ6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49217</v>
+        <v>49248</v>
       </c>
       <c r="DA6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49248</v>
+        <v>49278</v>
       </c>
       <c r="DB6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49278</v>
+        <v>49309</v>
       </c>
       <c r="DC6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49309</v>
+        <v>49340</v>
       </c>
       <c r="DD6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49340</v>
+        <v>49368</v>
       </c>
       <c r="DE6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49368</v>
+        <v>49399</v>
       </c>
       <c r="DF6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49399</v>
+        <v>49429</v>
       </c>
       <c r="DG6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49429</v>
+        <v>49460</v>
       </c>
       <c r="DH6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49460</v>
+        <v>49490</v>
       </c>
       <c r="DI6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49490</v>
+        <v>49521</v>
       </c>
       <c r="DJ6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49521</v>
+        <v>49552</v>
       </c>
       <c r="DK6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49552</v>
+        <v>49582</v>
       </c>
       <c r="DL6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49582</v>
+        <v>49613</v>
       </c>
       <c r="DM6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49613</v>
+        <v>49643</v>
       </c>
       <c r="DN6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49643</v>
+        <v>49674</v>
       </c>
       <c r="DO6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49674</v>
+        <v>49705</v>
       </c>
       <c r="DP6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49705</v>
+        <v>49734</v>
       </c>
       <c r="DQ6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49734</v>
+        <v>49765</v>
       </c>
       <c r="DR6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49765</v>
+        <v>49795</v>
       </c>
       <c r="DS6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49795</v>
+        <v>49826</v>
       </c>
       <c r="DT6" s="24">
         <f t="shared" ca="1" si="17"/>
-        <v>49826</v>
+        <v>49856</v>
       </c>
     </row>
     <row r="7" spans="2:124" x14ac:dyDescent="0.25">
@@ -13256,9 +13257,9 @@
         <f ca="1">-(J2*'Inputs &amp; Summary'!$D$68*(J3/1000))/12</f>
         <v>#VALUE!</v>
       </c>
-      <c r="K16" s="13" t="e">
+      <c r="K16" s="13">
         <f ca="1">-(K2*'Inputs &amp; Summary'!$D$68*(K3/1000))/12</f>
-        <v>#VALUE!</v>
+        <v>0</v>
       </c>
       <c r="L16" s="13">
         <f ca="1">-(L2*'Inputs &amp; Summary'!$D$68*(L3/1000))/12</f>
@@ -15675,7 +15676,7 @@
     </row>
     <row r="21" spans="2:124" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C21" s="32"/>
       <c r="D21" s="42">
@@ -28900,47 +28901,47 @@
       </c>
       <c r="C2" s="24">
         <f ca="1">'Inputs &amp; Summary'!$D$20</f>
-        <v>46170</v>
+        <v>46174</v>
       </c>
       <c r="D2" s="24">
         <f ca="1">EOMONTH(C2,12)</f>
-        <v>46538</v>
+        <v>46568</v>
       </c>
       <c r="E2" s="24">
         <f t="shared" ref="E2:M2" ca="1" si="0">EOMONTH(D2,12)</f>
-        <v>46904</v>
+        <v>46934</v>
       </c>
       <c r="F2" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>47269</v>
+        <v>47299</v>
       </c>
       <c r="G2" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>47634</v>
+        <v>47664</v>
       </c>
       <c r="H2" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>47999</v>
+        <v>48029</v>
       </c>
       <c r="I2" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>48365</v>
+        <v>48395</v>
       </c>
       <c r="J2" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>48730</v>
+        <v>48760</v>
       </c>
       <c r="K2" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>49095</v>
+        <v>49125</v>
       </c>
       <c r="L2" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>49460</v>
+        <v>49490</v>
       </c>
       <c r="M2" s="24">
         <f t="shared" ca="1" si="0"/>
-        <v>49826</v>
+        <v>49856</v>
       </c>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
@@ -29537,7 +29538,7 @@
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C16" s="42">
         <f>'Monthly Proforma'!D21</f>

</xml_diff>

<commit_message>
Added support for additional fields, improved testing, refactored main.py, updated README
</commit_message>
<xml_diff>
--- a/TCG Blank Model Template 2026-04-26.xlsx
+++ b/TCG Blank Model Template 2026-04-26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2434ef0feffdd206/Documents/Tryon Capital Group/Origination ^0 Due Diligence/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="739" documentId="13_ncr:1_{AF47EFD1-DEF7-4D96-959F-C8937757AD83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C50B14D-466A-42FD-9D20-0A8DA9F9853B}"/>
+  <xr:revisionPtr revIDLastSave="742" documentId="13_ncr:1_{AF47EFD1-DEF7-4D96-959F-C8937757AD83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C79AC225-EE1B-4DA9-B707-9F6D8DBC9B58}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,8 +28,10 @@
     <definedName name="AssessedValue">'Inputs &amp; Summary'!$D$70</definedName>
     <definedName name="Bathrooms">'Inputs &amp; Summary'!$D$9</definedName>
     <definedName name="Bedrooms">'Inputs &amp; Summary'!$D$8</definedName>
+    <definedName name="CityState">'Inputs &amp; Summary'!$D$4</definedName>
     <definedName name="ExpenseGrowth">'Inputs &amp; Summary'!$D$96</definedName>
     <definedName name="IncomeGrowth">'Inputs &amp; Summary'!$D$95</definedName>
+    <definedName name="InPlaceRent">'Inputs &amp; Summary'!$D$56</definedName>
     <definedName name="ListingDate">'Inputs &amp; Summary'!$D$5</definedName>
     <definedName name="LoanAmortization">'Inputs &amp; Summary'!$D$41</definedName>
     <definedName name="LoanAmount">'Inputs &amp; Summary'!$P$12</definedName>
@@ -39,6 +41,7 @@
     <definedName name="PurchasePrice">'Inputs &amp; Summary'!$D$17</definedName>
     <definedName name="ReassessmentFreq">'Inputs &amp; Summary'!$D$72</definedName>
     <definedName name="RentCastRent">'Inputs &amp; Summary'!$D$58</definedName>
+    <definedName name="SellerConcessions">'Inputs &amp; Summary'!$D$28</definedName>
     <definedName name="SquareFootage">'Inputs &amp; Summary'!$D$10</definedName>
     <definedName name="StreetAddress">'Inputs &amp; Summary'!$D$3</definedName>
     <definedName name="TaxValueAppreciation">'Inputs &amp; Summary'!$D$98</definedName>

</xml_diff>